<commit_message>
Admin corrigido e fluxo de importação validado
</commit_message>
<xml_diff>
--- a/importacoes/dados_empresas.xlsx
+++ b/importacoes/dados_empresas.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://arenabsbcombr-my.sharepoint.com/personal/joel_costa_arenabsb_com_br/Documents/Documentos/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-20.04\home\joelarena\sga\importacoes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3804C88B-C7B2-4F77-9FD5-988EAA57BB1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9CD3851-8B0C-40B5-938F-BF8784C9ABF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C916287A-9F0F-4F75-B4C3-78B46329AD1C}"/>
   </bookViews>

</xml_diff>